<commit_message>
Update CSP connect-src to include Groq and EMKC APIs, and update Selenium test reports
</commit_message>
<xml_diff>
--- a/test-cases-reports/selinium-test/selenium_web_report.xlsx
+++ b/test-cases-reports/selinium-test/selenium_web_report.xlsx
@@ -62,7 +62,7 @@
     <t>Total Duration</t>
   </si>
   <si>
-    <t>91.31s</t>
+    <t>90.58s</t>
   </si>
   <si>
     <t>Deployable Status</t>
@@ -92,7 +92,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>4.17s</t>
+    <t>4.32s</t>
   </si>
   <si>
     <t>-</t>
@@ -140,7 +140,7 @@
     <t>UI012: Onboarding page 3 title display</t>
   </si>
   <si>
-    <t>2.06s</t>
+    <t>2.11s</t>
   </si>
   <si>
     <t>UI013: Onboarding page 3 description text layout</t>
@@ -152,354 +152,354 @@
     <t>UI015: Login Screen background card shape</t>
   </si>
   <si>
-    <t>4.13s</t>
+    <t>4.12s</t>
   </si>
   <si>
     <t>UI016: Login screen email input container styling</t>
   </si>
   <si>
-    <t>4.16s</t>
-  </si>
-  <si>
     <t>UI017: Login screen password input container styling</t>
   </si>
   <si>
+    <t>UI018: Login button background design</t>
+  </si>
+  <si>
+    <t>UI019: Login header branding typography</t>
+  </si>
+  <si>
+    <t>UI020: Register screen fields typography and spacing</t>
+  </si>
+  <si>
+    <t>2.08s</t>
+  </si>
+  <si>
+    <t>UI021: Register button border radius</t>
+  </si>
+  <si>
+    <t>UI022: Register footer link styling</t>
+  </si>
+  <si>
+    <t>UI023: Bottom navigation bar alignment &amp; icon sets</t>
+  </si>
+  <si>
+    <t>UI024: Dashboard header title formatting</t>
+  </si>
+  <si>
+    <t>UI025: Theme toggler button visual contrast</t>
+  </si>
+  <si>
+    <t>UI026: Light mode dashboard theme colors</t>
+  </si>
+  <si>
+    <t>UI027: Dark mode theme transition styles</t>
+  </si>
+  <si>
+    <t>UI028: Profile screen user avatar size layout</t>
+  </si>
+  <si>
+    <t>UI029: Test session card border margins</t>
+  </si>
+  <si>
+    <t>UI030: AI Feedback dialog spacing layout</t>
+  </si>
+  <si>
+    <t>UI031: Onboarding page dot animation transition duration checks</t>
+  </si>
+  <si>
+    <t>UI032: Onboarding skip button typography style properties matching</t>
+  </si>
+  <si>
+    <t>UI033: Splash logo container dimensions ratio verification</t>
+  </si>
+  <si>
+    <t>UI034: Splash loader indicator circular progress thickness details</t>
+  </si>
+  <si>
+    <t>UI035: Authentication textfield error messaging text font style alignment</t>
+  </si>
+  <si>
+    <t>UI036: Login submit button responsive hover opacity changes</t>
+  </si>
+  <si>
+    <t>UI037: Register page input padding offsets consistency checks</t>
+  </si>
+  <si>
     <t>0.02s</t>
   </si>
   <si>
-    <t>UI018: Login button background design</t>
-  </si>
-  <si>
-    <t>UI019: Login header branding typography</t>
-  </si>
-  <si>
-    <t>UI020: Register screen fields typography and spacing</t>
+    <t>UI038: Custom appbar back navigation icon asset visual sizing</t>
+  </si>
+  <si>
+    <t>UI039: Dark mode active body background color matching parameters</t>
+  </si>
+  <si>
+    <t>UI040: Dashboard card shadows soft elevation border rendering</t>
+  </si>
+  <si>
+    <t>UI041: Tests tab bar category tab selected state visual highlight check</t>
+  </si>
+  <si>
+    <t>UI042: AI mock interview feedback container border lines styling</t>
+  </si>
+  <si>
+    <t>UI043: Chatbot user response chat bubble alignment properties</t>
+  </si>
+  <si>
+    <t>UI044: Chatbot assistant AI response bubble border radius constraints</t>
+  </si>
+  <si>
+    <t>UI045: Profile user name typography scale weight and contrast check</t>
+  </si>
+  <si>
+    <t>UI046: Settings theme toggle switch active color verification parameters</t>
+  </si>
+  <si>
+    <t>UI047: Onboarding title layout alignment centered checking</t>
+  </si>
+  <si>
+    <t>UI048: Textfields active cursor focus color validation</t>
+  </si>
+  <si>
+    <t>UI049: Error messages warning badge layout constraints</t>
+  </si>
+  <si>
+    <t>UI050: App notification icon badges count scaling parameters</t>
+  </si>
+  <si>
+    <t>UI051: Profile card statistics counts label typography sizing</t>
+  </si>
+  <si>
+    <t>UI052: HR round option button icons visual alignment</t>
+  </si>
+  <si>
+    <t>UI053: Tech round option card layout spacing check</t>
+  </si>
+  <si>
+    <t>UI054: Aptitude test category cards layout alignment parameters</t>
+  </si>
+  <si>
+    <t>UI055: Bottom sheet dialog header drag indicator bar styling</t>
+  </si>
+  <si>
+    <t>UI056: Alert dialog box overlay transparency index verification</t>
+  </si>
+  <si>
+    <t>UI057: Groq feedback score badge layout circular border alignment</t>
+  </si>
+  <si>
+    <t>UI058: Speech input icon active mic glow styling parameters</t>
+  </si>
+  <si>
+    <t>UI059: Dark theme input borders contrast rating validation</t>
+  </si>
+  <si>
+    <t>UI060: Onboarding next button icon placement side margins checking</t>
+  </si>
+  <si>
+    <t>UI061: Login form subtitle text wrapping behavior bounds verification</t>
+  </si>
+  <si>
+    <t>UI062: Profile layout scroll indicator visibility and design parameters</t>
+  </si>
+  <si>
+    <t>UI063: Aptitude quiz progress bar line color status verification</t>
+  </si>
+  <si>
+    <t>UI064: Custom card elements scaling values on larger resolutions</t>
+  </si>
+  <si>
+    <t>UI065: Custom list dividers height thickness checking parameters</t>
+  </si>
+  <si>
+    <t>UI066: Chat list loading skeleton screen layout alignment details</t>
+  </si>
+  <si>
+    <t>UI067: App header icon menu spacing and positioning specifications</t>
+  </si>
+  <si>
+    <t>UI068: Dialog dismiss button visual contrast and margin constraints</t>
+  </si>
+  <si>
+    <t>UI069: Text input fields placeholder character font styling rules</t>
+  </si>
+  <si>
+    <t>UI070: Feedback ratings star icons design grid layout parameters</t>
+  </si>
+  <si>
+    <t>UI071: Profile credentials edit inputs layout alignment values</t>
+  </si>
+  <si>
+    <t>UI072: Dashboard summary graphs axes labels readability scores check</t>
+  </si>
+  <si>
+    <t>UI073: Custom snackbar popup notifications container design styles</t>
+  </si>
+  <si>
+    <t>UI074: Speech to text helper guidelines panel visibility parameters</t>
+  </si>
+  <si>
+    <t>UI075: Webapp container shadow outline styling matching specifications</t>
+  </si>
+  <si>
+    <t>UI076: HR questions text wrapper paragraph line height constraints</t>
+  </si>
+  <si>
+    <t>UI077: Test score progress ring gauge indicator layout parameters</t>
+  </si>
+  <si>
+    <t>UI078: Dark theme headers shadow drop transitions layout options</t>
+  </si>
+  <si>
+    <t>UI079: Chat suggestion chips outline border thickness details</t>
+  </si>
+  <si>
+    <t>UI080: Settings section headers font size transformations checking</t>
+  </si>
+  <si>
+    <t>UI081: Login forgot password link visual underline toggle checks</t>
+  </si>
+  <si>
+    <t>UI082: Register legal policies agreements text box layouts checks</t>
+  </si>
+  <si>
+    <t>UI083: Placement details document viewer layout padding verification</t>
+  </si>
+  <si>
+    <t>UI084: Onboarding page transitions ease in curve validation limits</t>
+  </si>
+  <si>
+    <t>UI085: Custom dropdown selectors hover outline border width check</t>
+  </si>
+  <si>
+    <t>UI086: Dialog confirmations layouts check icon centering values</t>
+  </si>
+  <si>
+    <t>UI087: Chat input field icons click state opacity level updates</t>
+  </si>
+  <si>
+    <t>UI088: User avatar badge active placement online status display</t>
+  </si>
+  <si>
+    <t>UI089: Dashboard widgets responsive grid wrap breakpoint parameters</t>
+  </si>
+  <si>
+    <t>UI090: Error boundary layout screen logo styling matches guidelines</t>
+  </si>
+  <si>
+    <t>UI091: Aptitude result summary page visual headers scaling check</t>
+  </si>
+  <si>
+    <t>UI092: AI feedback details accordion expand collapse height values</t>
+  </si>
+  <si>
+    <t>UI093: Tech stack tags background pills color schemes mapping check</t>
+  </si>
+  <si>
+    <t>0.04s</t>
+  </si>
+  <si>
+    <t>UI094: Navigation bar labels selected font color parameter checks</t>
+  </si>
+  <si>
+    <t>UI095: Chat bot scroll to bottom button visual position layout</t>
+  </si>
+  <si>
+    <t>UI096: Settings section divider margins layout alignment specifications</t>
+  </si>
+  <si>
+    <t>UI097: Placement company filters panel layout drawer design styles</t>
+  </si>
+  <si>
+    <t>UI098: Notification toggle buttons sliding animation duration check</t>
+  </si>
+  <si>
+    <t>UI099: Onboarding screen 3 logo container height check bounds</t>
+  </si>
+  <si>
+    <t>UI100: Auth form title secondary text decoration attributes check</t>
+  </si>
+  <si>
+    <t>UI101: Chat message time badge indicator font weight properties</t>
+  </si>
+  <si>
+    <t>UI102: Profile page history entries list spacing parameters</t>
+  </si>
+  <si>
+    <t>UI103: Feedback text block alignment rules inside cards check</t>
+  </si>
+  <si>
+    <t>UI104: Custom tooltips hover dynamic layout rendering boundaries</t>
+  </si>
+  <si>
+    <t>UI105: Interview review card layout horizontal borders constraint</t>
+  </si>
+  <si>
+    <t>UI106: Light mode inputs focus border shadow layout checks</t>
+  </si>
+  <si>
+    <t>UI107: Settings clear cache option text style parameters matching</t>
+  </si>
+  <si>
+    <t>UI108: Placement job card badges layout visual check rules</t>
+  </si>
+  <si>
+    <t>UI109: Speech processing overlay spinner styling visual verification</t>
+  </si>
+  <si>
+    <t>UI110: Test report dashboard header title color styling verification</t>
+  </si>
+  <si>
+    <t>FN001: Load app page successfully</t>
+  </si>
+  <si>
+    <t>4.09s</t>
+  </si>
+  <si>
+    <t>FN002: Click Next to access page 2</t>
   </si>
   <si>
     <t>2.09s</t>
   </si>
   <si>
-    <t>UI021: Register button border radius</t>
-  </si>
-  <si>
-    <t>0.03s</t>
-  </si>
-  <si>
-    <t>UI022: Register footer link styling</t>
-  </si>
-  <si>
-    <t>UI023: Bottom navigation bar alignment &amp; icon sets</t>
-  </si>
-  <si>
-    <t>UI024: Dashboard header title formatting</t>
-  </si>
-  <si>
-    <t>UI025: Theme toggler button visual contrast</t>
-  </si>
-  <si>
-    <t>UI026: Light mode dashboard theme colors</t>
-  </si>
-  <si>
-    <t>UI027: Dark mode theme transition styles</t>
-  </si>
-  <si>
-    <t>UI028: Profile screen user avatar size layout</t>
-  </si>
-  <si>
-    <t>UI029: Test session card border margins</t>
-  </si>
-  <si>
-    <t>UI030: AI Feedback dialog spacing layout</t>
-  </si>
-  <si>
-    <t>UI031: Onboarding page dot animation transition duration checks</t>
-  </si>
-  <si>
-    <t>UI032: Onboarding skip button typography style properties matching</t>
-  </si>
-  <si>
-    <t>UI033: Splash logo container dimensions ratio verification</t>
-  </si>
-  <si>
-    <t>UI034: Splash loader indicator circular progress thickness details</t>
-  </si>
-  <si>
-    <t>UI035: Authentication textfield error messaging text font style alignment</t>
-  </si>
-  <si>
-    <t>UI036: Login submit button responsive hover opacity changes</t>
-  </si>
-  <si>
-    <t>UI037: Register page input padding offsets consistency checks</t>
-  </si>
-  <si>
-    <t>UI038: Custom appbar back navigation icon asset visual sizing</t>
-  </si>
-  <si>
-    <t>UI039: Dark mode active body background color matching parameters</t>
-  </si>
-  <si>
-    <t>UI040: Dashboard card shadows soft elevation border rendering</t>
-  </si>
-  <si>
-    <t>UI041: Tests tab bar category tab selected state visual highlight check</t>
-  </si>
-  <si>
-    <t>UI042: AI mock interview feedback container border lines styling</t>
-  </si>
-  <si>
-    <t>UI043: Chatbot user response chat bubble alignment properties</t>
-  </si>
-  <si>
-    <t>UI044: Chatbot assistant AI response bubble border radius constraints</t>
-  </si>
-  <si>
-    <t>UI045: Profile user name typography scale weight and contrast check</t>
-  </si>
-  <si>
-    <t>UI046: Settings theme toggle switch active color verification parameters</t>
-  </si>
-  <si>
-    <t>UI047: Onboarding title layout alignment centered checking</t>
-  </si>
-  <si>
-    <t>UI048: Textfields active cursor focus color validation</t>
-  </si>
-  <si>
-    <t>UI049: Error messages warning badge layout constraints</t>
-  </si>
-  <si>
-    <t>UI050: App notification icon badges count scaling parameters</t>
-  </si>
-  <si>
-    <t>UI051: Profile card statistics counts label typography sizing</t>
-  </si>
-  <si>
-    <t>UI052: HR round option button icons visual alignment</t>
-  </si>
-  <si>
-    <t>UI053: Tech round option card layout spacing check</t>
-  </si>
-  <si>
-    <t>UI054: Aptitude test category cards layout alignment parameters</t>
-  </si>
-  <si>
-    <t>UI055: Bottom sheet dialog header drag indicator bar styling</t>
-  </si>
-  <si>
-    <t>UI056: Alert dialog box overlay transparency index verification</t>
-  </si>
-  <si>
-    <t>UI057: Groq feedback score badge layout circular border alignment</t>
-  </si>
-  <si>
-    <t>UI058: Speech input icon active mic glow styling parameters</t>
-  </si>
-  <si>
-    <t>UI059: Dark theme input borders contrast rating validation</t>
-  </si>
-  <si>
-    <t>UI060: Onboarding next button icon placement side margins checking</t>
-  </si>
-  <si>
-    <t>UI061: Login form subtitle text wrapping behavior bounds verification</t>
-  </si>
-  <si>
-    <t>UI062: Profile layout scroll indicator visibility and design parameters</t>
-  </si>
-  <si>
-    <t>UI063: Aptitude quiz progress bar line color status verification</t>
-  </si>
-  <si>
-    <t>UI064: Custom card elements scaling values on larger resolutions</t>
-  </si>
-  <si>
-    <t>UI065: Custom list dividers height thickness checking parameters</t>
-  </si>
-  <si>
-    <t>UI066: Chat list loading skeleton screen layout alignment details</t>
-  </si>
-  <si>
-    <t>UI067: App header icon menu spacing and positioning specifications</t>
-  </si>
-  <si>
-    <t>UI068: Dialog dismiss button visual contrast and margin constraints</t>
-  </si>
-  <si>
-    <t>UI069: Text input fields placeholder character font styling rules</t>
-  </si>
-  <si>
-    <t>UI070: Feedback ratings star icons design grid layout parameters</t>
-  </si>
-  <si>
-    <t>UI071: Profile credentials edit inputs layout alignment values</t>
-  </si>
-  <si>
-    <t>UI072: Dashboard summary graphs axes labels readability scores check</t>
-  </si>
-  <si>
-    <t>UI073: Custom snackbar popup notifications container design styles</t>
-  </si>
-  <si>
-    <t>UI074: Speech to text helper guidelines panel visibility parameters</t>
-  </si>
-  <si>
-    <t>UI075: Webapp container shadow outline styling matching specifications</t>
-  </si>
-  <si>
-    <t>UI076: HR questions text wrapper paragraph line height constraints</t>
-  </si>
-  <si>
-    <t>UI077: Test score progress ring gauge indicator layout parameters</t>
-  </si>
-  <si>
-    <t>UI078: Dark theme headers shadow drop transitions layout options</t>
-  </si>
-  <si>
-    <t>UI079: Chat suggestion chips outline border thickness details</t>
-  </si>
-  <si>
-    <t>UI080: Settings section headers font size transformations checking</t>
-  </si>
-  <si>
-    <t>UI081: Login forgot password link visual underline toggle checks</t>
-  </si>
-  <si>
-    <t>UI082: Register legal policies agreements text box layouts checks</t>
-  </si>
-  <si>
-    <t>UI083: Placement details document viewer layout padding verification</t>
-  </si>
-  <si>
-    <t>UI084: Onboarding page transitions ease in curve validation limits</t>
-  </si>
-  <si>
-    <t>UI085: Custom dropdown selectors hover outline border width check</t>
-  </si>
-  <si>
-    <t>UI086: Dialog confirmations layouts check icon centering values</t>
-  </si>
-  <si>
-    <t>UI087: Chat input field icons click state opacity level updates</t>
-  </si>
-  <si>
-    <t>UI088: User avatar badge active placement online status display</t>
-  </si>
-  <si>
-    <t>UI089: Dashboard widgets responsive grid wrap breakpoint parameters</t>
-  </si>
-  <si>
-    <t>UI090: Error boundary layout screen logo styling matches guidelines</t>
-  </si>
-  <si>
-    <t>UI091: Aptitude result summary page visual headers scaling check</t>
-  </si>
-  <si>
-    <t>UI092: AI feedback details accordion expand collapse height values</t>
-  </si>
-  <si>
-    <t>UI093: Tech stack tags background pills color schemes mapping check</t>
-  </si>
-  <si>
-    <t>UI094: Navigation bar labels selected font color parameter checks</t>
-  </si>
-  <si>
-    <t>UI095: Chat bot scroll to bottom button visual position layout</t>
-  </si>
-  <si>
-    <t>UI096: Settings section divider margins layout alignment specifications</t>
-  </si>
-  <si>
-    <t>UI097: Placement company filters panel layout drawer design styles</t>
-  </si>
-  <si>
-    <t>UI098: Notification toggle buttons sliding animation duration check</t>
-  </si>
-  <si>
-    <t>UI099: Onboarding screen 3 logo container height check bounds</t>
-  </si>
-  <si>
-    <t>UI100: Auth form title secondary text decoration attributes check</t>
-  </si>
-  <si>
-    <t>UI101: Chat message time badge indicator font weight properties</t>
-  </si>
-  <si>
-    <t>UI102: Profile page history entries list spacing parameters</t>
-  </si>
-  <si>
-    <t>UI103: Feedback text block alignment rules inside cards check</t>
-  </si>
-  <si>
-    <t>UI104: Custom tooltips hover dynamic layout rendering boundaries</t>
-  </si>
-  <si>
-    <t>0.04s</t>
-  </si>
-  <si>
-    <t>UI105: Interview review card layout horizontal borders constraint</t>
-  </si>
-  <si>
-    <t>UI106: Light mode inputs focus border shadow layout checks</t>
-  </si>
-  <si>
-    <t>UI107: Settings clear cache option text style parameters matching</t>
-  </si>
-  <si>
-    <t>UI108: Placement job card badges layout visual check rules</t>
-  </si>
-  <si>
-    <t>UI109: Speech processing overlay spinner styling visual verification</t>
-  </si>
-  <si>
-    <t>UI110: Test report dashboard header title color styling verification</t>
-  </si>
-  <si>
-    <t>FN001: Load app page successfully</t>
-  </si>
-  <si>
-    <t>FN002: Click Next to access page 2</t>
+    <t>FN003: Click Next to access page 3</t>
+  </si>
+  <si>
+    <t>FN004: Skip button bypasses onboarding screen</t>
+  </si>
+  <si>
+    <t>6.17s</t>
+  </si>
+  <si>
+    <t>FN005: Complete onboarding and transition to authentication page</t>
+  </si>
+  <si>
+    <t>2.13s</t>
+  </si>
+  <si>
+    <t>FN006: Select register navigation path</t>
+  </si>
+  <si>
+    <t>FN007: Register a new account with valid unique details</t>
+  </si>
+  <si>
+    <t>FN008: Submit register account credentials to Firestore</t>
   </si>
   <si>
     <t>2.07s</t>
   </si>
   <si>
-    <t>FN003: Click Next to access page 3</t>
-  </si>
-  <si>
-    <t>2.08s</t>
-  </si>
-  <si>
-    <t>FN004: Skip button bypasses onboarding screen</t>
-  </si>
-  <si>
-    <t>6.24s</t>
-  </si>
-  <si>
-    <t>FN005: Complete onboarding and transition to authentication page</t>
-  </si>
-  <si>
-    <t>FN006: Select register navigation path</t>
-  </si>
-  <si>
-    <t>2.11s</t>
-  </si>
-  <si>
-    <t>FN007: Register a new account with valid unique details</t>
-  </si>
-  <si>
-    <t>FN008: Submit register account credentials to Firestore</t>
-  </si>
-  <si>
     <t>FN009: Verify user main dashboard is successfully loaded</t>
   </si>
   <si>
-    <t>0.54s</t>
+    <t>0.53s</t>
   </si>
   <si>
     <t>FN010: Navigate to Aptitude &amp; Technical Tests tab</t>
   </si>
   <si>
+    <t>2.12s</t>
+  </si>
+  <si>
     <t>FN011: Render Aptitude list categories</t>
   </si>
   <si>
@@ -530,37 +530,40 @@
     <t>FN019: Input answer to the generated mock question</t>
   </si>
   <si>
+    <t>4.19s</t>
+  </si>
+  <si>
+    <t>FN020: Submit answer to AI evaluation engine</t>
+  </si>
+  <si>
+    <t>FN021: Retrieve feedback score from Groq API response</t>
+  </si>
+  <si>
+    <t>2.01s</t>
+  </si>
+  <si>
+    <t>FN022: Display evaluation advice layout</t>
+  </si>
+  <si>
+    <t>FN023: Exit active interview page using close option</t>
+  </si>
+  <si>
+    <t>FN024: Exit dialog confirmation redirects back to dashboard</t>
+  </si>
+  <si>
+    <t>FN025: Navigate to Chatbot assistant tab</t>
+  </si>
+  <si>
+    <t>FN026: Enter custom text message in chat query input</t>
+  </si>
+  <si>
     <t>4.18s</t>
   </si>
   <si>
-    <t>FN020: Submit answer to AI evaluation engine</t>
-  </si>
-  <si>
-    <t>FN021: Retrieve feedback score from Groq API response</t>
-  </si>
-  <si>
-    <t>2.03s</t>
-  </si>
-  <si>
-    <t>FN022: Display evaluation advice layout</t>
-  </si>
-  <si>
-    <t>FN023: Exit active interview page using close option</t>
-  </si>
-  <si>
-    <t>FN024: Exit dialog confirmation redirects back to dashboard</t>
-  </si>
-  <si>
-    <t>FN025: Navigate to Chatbot assistant tab</t>
-  </si>
-  <si>
-    <t>FN026: Enter custom text message in chat query input</t>
-  </si>
-  <si>
     <t>FN027: Receive chatbot answer correctly</t>
   </si>
   <si>
-    <t>1.01s</t>
+    <t>1.04s</t>
   </si>
   <si>
     <t>FN028: Access user settings &amp; profile tab</t>
@@ -1121,39 +1124,39 @@
     <t>VL002: Register user empty last name triggers validation</t>
   </si>
   <si>
+    <t>VL003: Register user blank email validation toast</t>
+  </si>
+  <si>
+    <t>VL004: Register user invalid email format display</t>
+  </si>
+  <si>
+    <t>VL005: Register user weak password complexity warning display</t>
+  </si>
+  <si>
+    <t>VL006: Authenticate with invalid email formatting</t>
+  </si>
+  <si>
+    <t>VL007: Authenticate with wrong password key error toast</t>
+  </si>
+  <si>
+    <t>0.12s</t>
+  </si>
+  <si>
+    <t>VL008: Submit empty text answer to HR Interviewer returns validation message</t>
+  </si>
+  <si>
+    <t>VL009: Check question counts upper limit constraint</t>
+  </si>
+  <si>
+    <t>VL010: Check question counts lower limit constraint</t>
+  </si>
+  <si>
+    <t>VL011: Submit aptitude test with no questions answered displays alert dialog</t>
+  </si>
+  <si>
     <t>0.10s</t>
   </si>
   <si>
-    <t>VL003: Register user blank email validation toast</t>
-  </si>
-  <si>
-    <t>0.12s</t>
-  </si>
-  <si>
-    <t>VL004: Register user invalid email format display</t>
-  </si>
-  <si>
-    <t>VL005: Register user weak password complexity warning display</t>
-  </si>
-  <si>
-    <t>VL006: Authenticate with invalid email formatting</t>
-  </si>
-  <si>
-    <t>VL007: Authenticate with wrong password key error toast</t>
-  </si>
-  <si>
-    <t>VL008: Submit empty text answer to HR Interviewer returns validation message</t>
-  </si>
-  <si>
-    <t>VL009: Check question counts upper limit constraint</t>
-  </si>
-  <si>
-    <t>VL010: Check question counts lower limit constraint</t>
-  </si>
-  <si>
-    <t>VL011: Submit aptitude test with no questions answered displays alert dialog</t>
-  </si>
-  <si>
     <t>VL012: Save offline test session log validation check</t>
   </si>
   <si>
@@ -1272,9 +1275,6 @@
   </si>
   <si>
     <t>VL051: Auth token formats validation checks matches regex syntax rules</t>
-  </si>
-  <si>
-    <t>0.05s</t>
   </si>
   <si>
     <t>VL052: Custom dashboard stats metrics numerical constraints boundaries</t>
@@ -2232,7 +2232,7 @@
         <v>25</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>27</v>
@@ -2334,7 +2334,7 @@
         <v>25</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>27</v>
@@ -2345,13 +2345,13 @@
         <v>7</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>27</v>
@@ -2362,13 +2362,13 @@
         <v>7</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>27</v>
@@ -2379,7 +2379,7 @@
         <v>7</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>25</v>
@@ -2396,13 +2396,13 @@
         <v>7</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>27</v>
@@ -2413,13 +2413,13 @@
         <v>7</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C22" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="E22" s="10" t="s">
         <v>27</v>
@@ -2430,7 +2430,7 @@
         <v>7</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>25</v>
@@ -2447,7 +2447,7 @@
         <v>7</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C24" s="11" t="s">
         <v>25</v>
@@ -2464,7 +2464,7 @@
         <v>7</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>25</v>
@@ -2481,7 +2481,7 @@
         <v>7</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>25</v>
@@ -2498,7 +2498,7 @@
         <v>7</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>25</v>
@@ -2515,7 +2515,7 @@
         <v>7</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>25</v>
@@ -2532,7 +2532,7 @@
         <v>7</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>25</v>
@@ -2549,7 +2549,7 @@
         <v>7</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>25</v>
@@ -2566,7 +2566,7 @@
         <v>7</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>25</v>
@@ -2583,7 +2583,7 @@
         <v>7</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>25</v>
@@ -2600,7 +2600,7 @@
         <v>7</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>25</v>
@@ -2617,7 +2617,7 @@
         <v>7</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>25</v>
@@ -2634,7 +2634,7 @@
         <v>7</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>25</v>
@@ -2651,7 +2651,7 @@
         <v>7</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>25</v>
@@ -2668,13 +2668,13 @@
         <v>7</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>27</v>
@@ -2685,13 +2685,13 @@
         <v>7</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="E38" s="10" t="s">
         <v>27</v>
@@ -2702,7 +2702,7 @@
         <v>7</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>25</v>
@@ -2719,7 +2719,7 @@
         <v>7</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C40" s="11" t="s">
         <v>25</v>
@@ -2736,7 +2736,7 @@
         <v>7</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C41" s="11" t="s">
         <v>25</v>
@@ -2753,7 +2753,7 @@
         <v>7</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C42" s="11" t="s">
         <v>25</v>
@@ -2770,7 +2770,7 @@
         <v>7</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C43" s="11" t="s">
         <v>25</v>
@@ -2787,7 +2787,7 @@
         <v>7</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C44" s="11" t="s">
         <v>25</v>
@@ -2804,7 +2804,7 @@
         <v>7</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C45" s="11" t="s">
         <v>25</v>
@@ -2821,7 +2821,7 @@
         <v>7</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C46" s="11" t="s">
         <v>25</v>
@@ -2838,7 +2838,7 @@
         <v>7</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C47" s="11" t="s">
         <v>25</v>
@@ -2855,7 +2855,7 @@
         <v>7</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C48" s="11" t="s">
         <v>25</v>
@@ -2872,7 +2872,7 @@
         <v>7</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C49" s="11" t="s">
         <v>25</v>
@@ -2889,7 +2889,7 @@
         <v>7</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C50" s="11" t="s">
         <v>25</v>
@@ -2906,7 +2906,7 @@
         <v>7</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C51" s="11" t="s">
         <v>25</v>
@@ -2923,7 +2923,7 @@
         <v>7</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C52" s="11" t="s">
         <v>25</v>
@@ -2940,7 +2940,7 @@
         <v>7</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C53" s="11" t="s">
         <v>25</v>
@@ -2957,7 +2957,7 @@
         <v>7</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C54" s="11" t="s">
         <v>25</v>
@@ -2974,7 +2974,7 @@
         <v>7</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C55" s="11" t="s">
         <v>25</v>
@@ -2991,7 +2991,7 @@
         <v>7</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C56" s="11" t="s">
         <v>25</v>
@@ -3008,7 +3008,7 @@
         <v>7</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C57" s="11" t="s">
         <v>25</v>
@@ -3025,7 +3025,7 @@
         <v>7</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C58" s="11" t="s">
         <v>25</v>
@@ -3042,7 +3042,7 @@
         <v>7</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C59" s="11" t="s">
         <v>25</v>
@@ -3059,7 +3059,7 @@
         <v>7</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C60" s="11" t="s">
         <v>25</v>
@@ -3076,7 +3076,7 @@
         <v>7</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C61" s="11" t="s">
         <v>25</v>
@@ -3093,7 +3093,7 @@
         <v>7</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C62" s="11" t="s">
         <v>25</v>
@@ -3110,7 +3110,7 @@
         <v>7</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C63" s="11" t="s">
         <v>25</v>
@@ -3127,7 +3127,7 @@
         <v>7</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C64" s="11" t="s">
         <v>25</v>
@@ -3144,7 +3144,7 @@
         <v>7</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C65" s="11" t="s">
         <v>25</v>
@@ -3161,7 +3161,7 @@
         <v>7</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C66" s="11" t="s">
         <v>25</v>
@@ -3178,7 +3178,7 @@
         <v>7</v>
       </c>
       <c r="B67" s="10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C67" s="11" t="s">
         <v>25</v>
@@ -3195,7 +3195,7 @@
         <v>7</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C68" s="11" t="s">
         <v>25</v>
@@ -3212,7 +3212,7 @@
         <v>7</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C69" s="11" t="s">
         <v>25</v>
@@ -3229,7 +3229,7 @@
         <v>7</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C70" s="11" t="s">
         <v>25</v>
@@ -3246,7 +3246,7 @@
         <v>7</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C71" s="11" t="s">
         <v>25</v>
@@ -3263,7 +3263,7 @@
         <v>7</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C72" s="11" t="s">
         <v>25</v>
@@ -3280,7 +3280,7 @@
         <v>7</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C73" s="11" t="s">
         <v>25</v>
@@ -3297,7 +3297,7 @@
         <v>7</v>
       </c>
       <c r="B74" s="10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C74" s="11" t="s">
         <v>25</v>
@@ -3314,7 +3314,7 @@
         <v>7</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C75" s="11" t="s">
         <v>25</v>
@@ -3331,7 +3331,7 @@
         <v>7</v>
       </c>
       <c r="B76" s="10" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C76" s="11" t="s">
         <v>25</v>
@@ -3348,7 +3348,7 @@
         <v>7</v>
       </c>
       <c r="B77" s="10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C77" s="11" t="s">
         <v>25</v>
@@ -3365,7 +3365,7 @@
         <v>7</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C78" s="11" t="s">
         <v>25</v>
@@ -3382,7 +3382,7 @@
         <v>7</v>
       </c>
       <c r="B79" s="10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C79" s="11" t="s">
         <v>25</v>
@@ -3399,7 +3399,7 @@
         <v>7</v>
       </c>
       <c r="B80" s="10" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C80" s="11" t="s">
         <v>25</v>
@@ -3416,7 +3416,7 @@
         <v>7</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C81" s="11" t="s">
         <v>25</v>
@@ -3433,7 +3433,7 @@
         <v>7</v>
       </c>
       <c r="B82" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C82" s="11" t="s">
         <v>25</v>
@@ -3450,7 +3450,7 @@
         <v>7</v>
       </c>
       <c r="B83" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C83" s="11" t="s">
         <v>25</v>
@@ -3467,7 +3467,7 @@
         <v>7</v>
       </c>
       <c r="B84" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C84" s="11" t="s">
         <v>25</v>
@@ -3484,7 +3484,7 @@
         <v>7</v>
       </c>
       <c r="B85" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C85" s="11" t="s">
         <v>25</v>
@@ -3501,7 +3501,7 @@
         <v>7</v>
       </c>
       <c r="B86" s="10" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C86" s="11" t="s">
         <v>25</v>
@@ -3518,7 +3518,7 @@
         <v>7</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C87" s="11" t="s">
         <v>25</v>
@@ -3535,7 +3535,7 @@
         <v>7</v>
       </c>
       <c r="B88" s="10" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C88" s="11" t="s">
         <v>25</v>
@@ -3552,7 +3552,7 @@
         <v>7</v>
       </c>
       <c r="B89" s="10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C89" s="11" t="s">
         <v>25</v>
@@ -3569,7 +3569,7 @@
         <v>7</v>
       </c>
       <c r="B90" s="10" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C90" s="11" t="s">
         <v>25</v>
@@ -3586,7 +3586,7 @@
         <v>7</v>
       </c>
       <c r="B91" s="10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C91" s="11" t="s">
         <v>25</v>
@@ -3603,7 +3603,7 @@
         <v>7</v>
       </c>
       <c r="B92" s="10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C92" s="11" t="s">
         <v>25</v>
@@ -3620,7 +3620,7 @@
         <v>7</v>
       </c>
       <c r="B93" s="10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C93" s="11" t="s">
         <v>25</v>
@@ -3637,13 +3637,13 @@
         <v>7</v>
       </c>
       <c r="B94" s="10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C94" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D94" s="12" t="s">
-        <v>29</v>
+        <v>127</v>
       </c>
       <c r="E94" s="10" t="s">
         <v>27</v>
@@ -3654,7 +3654,7 @@
         <v>7</v>
       </c>
       <c r="B95" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C95" s="11" t="s">
         <v>25</v>
@@ -3671,7 +3671,7 @@
         <v>7</v>
       </c>
       <c r="B96" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C96" s="11" t="s">
         <v>25</v>
@@ -3688,7 +3688,7 @@
         <v>7</v>
       </c>
       <c r="B97" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C97" s="11" t="s">
         <v>25</v>
@@ -3705,7 +3705,7 @@
         <v>7</v>
       </c>
       <c r="B98" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C98" s="11" t="s">
         <v>25</v>
@@ -3722,7 +3722,7 @@
         <v>7</v>
       </c>
       <c r="B99" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C99" s="11" t="s">
         <v>25</v>
@@ -3739,13 +3739,13 @@
         <v>7</v>
       </c>
       <c r="B100" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C100" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D100" s="12" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="E100" s="10" t="s">
         <v>27</v>
@@ -3756,7 +3756,7 @@
         <v>7</v>
       </c>
       <c r="B101" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C101" s="11" t="s">
         <v>25</v>
@@ -3773,7 +3773,7 @@
         <v>7</v>
       </c>
       <c r="B102" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C102" s="11" t="s">
         <v>25</v>
@@ -3790,13 +3790,13 @@
         <v>7</v>
       </c>
       <c r="B103" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C103" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D103" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E103" s="10" t="s">
         <v>27</v>
@@ -3807,13 +3807,13 @@
         <v>7</v>
       </c>
       <c r="B104" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C104" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D104" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E104" s="10" t="s">
         <v>27</v>
@@ -3824,13 +3824,13 @@
         <v>7</v>
       </c>
       <c r="B105" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C105" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D105" s="12" t="s">
-        <v>140</v>
+        <v>29</v>
       </c>
       <c r="E105" s="10" t="s">
         <v>27</v>
@@ -3841,7 +3841,7 @@
         <v>7</v>
       </c>
       <c r="B106" s="10" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C106" s="11" t="s">
         <v>25</v>
@@ -3858,13 +3858,13 @@
         <v>7</v>
       </c>
       <c r="B107" s="10" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C107" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D107" s="12" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="E107" s="10" t="s">
         <v>27</v>
@@ -3875,7 +3875,7 @@
         <v>7</v>
       </c>
       <c r="B108" s="10" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C108" s="11" t="s">
         <v>25</v>
@@ -3892,7 +3892,7 @@
         <v>7</v>
       </c>
       <c r="B109" s="10" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C109" s="11" t="s">
         <v>25</v>
@@ -3909,7 +3909,7 @@
         <v>7</v>
       </c>
       <c r="B110" s="10" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C110" s="11" t="s">
         <v>25</v>
@@ -3926,7 +3926,7 @@
         <v>7</v>
       </c>
       <c r="B111" s="10" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C111" s="11" t="s">
         <v>25</v>
@@ -3943,13 +3943,13 @@
         <v>10</v>
       </c>
       <c r="B112" s="10" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C112" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D112" s="12" t="s">
-        <v>46</v>
+        <v>146</v>
       </c>
       <c r="E112" s="10" t="s">
         <v>27</v>
@@ -3960,13 +3960,13 @@
         <v>10</v>
       </c>
       <c r="B113" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="C113" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D113" s="12" t="s">
         <v>148</v>
-      </c>
-      <c r="C113" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="D113" s="12" t="s">
-        <v>149</v>
       </c>
       <c r="E113" s="10" t="s">
         <v>27</v>
@@ -3977,13 +3977,13 @@
         <v>10</v>
       </c>
       <c r="B114" s="10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C114" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D114" s="12" t="s">
-        <v>151</v>
+        <v>42</v>
       </c>
       <c r="E114" s="10" t="s">
         <v>27</v>
@@ -3994,13 +3994,13 @@
         <v>10</v>
       </c>
       <c r="B115" s="10" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C115" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D115" s="12" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E115" s="10" t="s">
         <v>27</v>
@@ -4011,13 +4011,13 @@
         <v>10</v>
       </c>
       <c r="B116" s="10" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C116" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D116" s="12" t="s">
-        <v>54</v>
+        <v>153</v>
       </c>
       <c r="E116" s="10" t="s">
         <v>27</v>
@@ -4028,13 +4028,13 @@
         <v>10</v>
       </c>
       <c r="B117" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C117" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D117" s="12" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="E117" s="10" t="s">
         <v>27</v>
@@ -4045,13 +4045,13 @@
         <v>10</v>
       </c>
       <c r="B118" s="10" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C118" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D118" s="12" t="s">
-        <v>38</v>
+        <v>148</v>
       </c>
       <c r="E118" s="10" t="s">
         <v>27</v>
@@ -4062,13 +4062,13 @@
         <v>10</v>
       </c>
       <c r="B119" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C119" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D119" s="12" t="s">
-        <v>38</v>
+        <v>157</v>
       </c>
       <c r="E119" s="10" t="s">
         <v>27</v>
@@ -4079,13 +4079,13 @@
         <v>10</v>
       </c>
       <c r="B120" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="C120" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D120" s="12" t="s">
         <v>159</v>
-      </c>
-      <c r="C120" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="D120" s="12" t="s">
-        <v>160</v>
       </c>
       <c r="E120" s="10" t="s">
         <v>27</v>
@@ -4096,13 +4096,13 @@
         <v>10</v>
       </c>
       <c r="B121" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="C121" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D121" s="12" t="s">
         <v>161</v>
-      </c>
-      <c r="C121" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="D121" s="12" t="s">
-        <v>156</v>
       </c>
       <c r="E121" s="10" t="s">
         <v>27</v>
@@ -4136,7 +4136,7 @@
         <v>25</v>
       </c>
       <c r="D123" s="12" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="E123" s="10" t="s">
         <v>27</v>
@@ -4153,7 +4153,7 @@
         <v>25</v>
       </c>
       <c r="D124" s="12" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="E124" s="10" t="s">
         <v>27</v>
@@ -4170,7 +4170,7 @@
         <v>25</v>
       </c>
       <c r="D125" s="12" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E125" s="10" t="s">
         <v>27</v>
@@ -4187,7 +4187,7 @@
         <v>25</v>
       </c>
       <c r="D126" s="12" t="s">
-        <v>54</v>
+        <v>157</v>
       </c>
       <c r="E126" s="10" t="s">
         <v>27</v>
@@ -4204,7 +4204,7 @@
         <v>25</v>
       </c>
       <c r="D127" s="12" t="s">
-        <v>156</v>
+        <v>52</v>
       </c>
       <c r="E127" s="10" t="s">
         <v>27</v>
@@ -4238,7 +4238,7 @@
         <v>25</v>
       </c>
       <c r="D129" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E129" s="10" t="s">
         <v>27</v>
@@ -4272,7 +4272,7 @@
         <v>25</v>
       </c>
       <c r="D131" s="12" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="E131" s="10" t="s">
         <v>27</v>
@@ -4306,7 +4306,7 @@
         <v>25</v>
       </c>
       <c r="D133" s="12" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E133" s="10" t="s">
         <v>27</v>
@@ -4323,7 +4323,7 @@
         <v>25</v>
       </c>
       <c r="D134" s="12" t="s">
-        <v>151</v>
+        <v>52</v>
       </c>
       <c r="E134" s="10" t="s">
         <v>27</v>
@@ -4340,7 +4340,7 @@
         <v>25</v>
       </c>
       <c r="D135" s="12" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E135" s="10" t="s">
         <v>27</v>
@@ -4357,7 +4357,7 @@
         <v>25</v>
       </c>
       <c r="D136" s="12" t="s">
-        <v>54</v>
+        <v>153</v>
       </c>
       <c r="E136" s="10" t="s">
         <v>27</v>
@@ -4374,7 +4374,7 @@
         <v>25</v>
       </c>
       <c r="D137" s="12" t="s">
-        <v>26</v>
+        <v>181</v>
       </c>
       <c r="E137" s="10" t="s">
         <v>27</v>
@@ -4385,13 +4385,13 @@
         <v>10</v>
       </c>
       <c r="B138" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C138" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D138" s="12" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E138" s="10" t="s">
         <v>27</v>
@@ -4402,13 +4402,13 @@
         <v>10</v>
       </c>
       <c r="B139" s="10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C139" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D139" s="12" t="s">
-        <v>156</v>
+        <v>38</v>
       </c>
       <c r="E139" s="10" t="s">
         <v>27</v>
@@ -4419,13 +4419,13 @@
         <v>10</v>
       </c>
       <c r="B140" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C140" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D140" s="12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E140" s="10" t="s">
         <v>27</v>
@@ -4436,13 +4436,13 @@
         <v>10</v>
       </c>
       <c r="B141" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C141" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D141" s="12" t="s">
-        <v>54</v>
+        <v>161</v>
       </c>
       <c r="E141" s="10" t="s">
         <v>27</v>
@@ -4453,7 +4453,7 @@
         <v>10</v>
       </c>
       <c r="B142" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C142" s="11" t="s">
         <v>25</v>
@@ -4470,7 +4470,7 @@
         <v>10</v>
       </c>
       <c r="B143" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C143" s="11" t="s">
         <v>25</v>
@@ -4487,7 +4487,7 @@
         <v>10</v>
       </c>
       <c r="B144" s="10" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C144" s="11" t="s">
         <v>25</v>
@@ -4504,7 +4504,7 @@
         <v>10</v>
       </c>
       <c r="B145" s="10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C145" s="11" t="s">
         <v>25</v>
@@ -4521,7 +4521,7 @@
         <v>10</v>
       </c>
       <c r="B146" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C146" s="11" t="s">
         <v>25</v>
@@ -4538,7 +4538,7 @@
         <v>10</v>
       </c>
       <c r="B147" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C147" s="11" t="s">
         <v>25</v>
@@ -4555,7 +4555,7 @@
         <v>10</v>
       </c>
       <c r="B148" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C148" s="11" t="s">
         <v>25</v>
@@ -4572,7 +4572,7 @@
         <v>10</v>
       </c>
       <c r="B149" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C149" s="11" t="s">
         <v>25</v>
@@ -4589,13 +4589,13 @@
         <v>10</v>
       </c>
       <c r="B150" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C150" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D150" s="12" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E150" s="10" t="s">
         <v>27</v>
@@ -4606,7 +4606,7 @@
         <v>10</v>
       </c>
       <c r="B151" s="10" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C151" s="11" t="s">
         <v>25</v>
@@ -4623,7 +4623,7 @@
         <v>10</v>
       </c>
       <c r="B152" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C152" s="11" t="s">
         <v>25</v>
@@ -4640,7 +4640,7 @@
         <v>10</v>
       </c>
       <c r="B153" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C153" s="11" t="s">
         <v>25</v>
@@ -4657,7 +4657,7 @@
         <v>10</v>
       </c>
       <c r="B154" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C154" s="11" t="s">
         <v>25</v>
@@ -4674,7 +4674,7 @@
         <v>10</v>
       </c>
       <c r="B155" s="10" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C155" s="11" t="s">
         <v>25</v>
@@ -4691,7 +4691,7 @@
         <v>10</v>
       </c>
       <c r="B156" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C156" s="11" t="s">
         <v>25</v>
@@ -4708,7 +4708,7 @@
         <v>10</v>
       </c>
       <c r="B157" s="10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C157" s="11" t="s">
         <v>25</v>
@@ -4725,7 +4725,7 @@
         <v>10</v>
       </c>
       <c r="B158" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C158" s="11" t="s">
         <v>25</v>
@@ -4742,7 +4742,7 @@
         <v>10</v>
       </c>
       <c r="B159" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C159" s="11" t="s">
         <v>25</v>
@@ -4759,13 +4759,13 @@
         <v>10</v>
       </c>
       <c r="B160" s="10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C160" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D160" s="12" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E160" s="10" t="s">
         <v>27</v>
@@ -4776,7 +4776,7 @@
         <v>10</v>
       </c>
       <c r="B161" s="10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C161" s="11" t="s">
         <v>25</v>
@@ -4793,7 +4793,7 @@
         <v>10</v>
       </c>
       <c r="B162" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C162" s="11" t="s">
         <v>25</v>
@@ -4810,7 +4810,7 @@
         <v>10</v>
       </c>
       <c r="B163" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C163" s="11" t="s">
         <v>25</v>
@@ -4827,7 +4827,7 @@
         <v>10</v>
       </c>
       <c r="B164" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C164" s="11" t="s">
         <v>25</v>
@@ -4844,7 +4844,7 @@
         <v>10</v>
       </c>
       <c r="B165" s="10" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C165" s="11" t="s">
         <v>25</v>
@@ -4861,7 +4861,7 @@
         <v>10</v>
       </c>
       <c r="B166" s="10" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C166" s="11" t="s">
         <v>25</v>
@@ -4878,7 +4878,7 @@
         <v>10</v>
       </c>
       <c r="B167" s="10" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C167" s="11" t="s">
         <v>25</v>
@@ -4895,7 +4895,7 @@
         <v>10</v>
       </c>
       <c r="B168" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C168" s="11" t="s">
         <v>25</v>
@@ -4912,7 +4912,7 @@
         <v>10</v>
       </c>
       <c r="B169" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C169" s="11" t="s">
         <v>25</v>
@@ -4929,7 +4929,7 @@
         <v>10</v>
       </c>
       <c r="B170" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C170" s="11" t="s">
         <v>25</v>
@@ -4946,7 +4946,7 @@
         <v>10</v>
       </c>
       <c r="B171" s="10" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C171" s="11" t="s">
         <v>25</v>
@@ -4963,7 +4963,7 @@
         <v>10</v>
       </c>
       <c r="B172" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C172" s="11" t="s">
         <v>25</v>
@@ -4980,7 +4980,7 @@
         <v>10</v>
       </c>
       <c r="B173" s="10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C173" s="11" t="s">
         <v>25</v>
@@ -4997,7 +4997,7 @@
         <v>10</v>
       </c>
       <c r="B174" s="10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C174" s="11" t="s">
         <v>25</v>
@@ -5014,7 +5014,7 @@
         <v>10</v>
       </c>
       <c r="B175" s="10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C175" s="11" t="s">
         <v>25</v>
@@ -5031,7 +5031,7 @@
         <v>10</v>
       </c>
       <c r="B176" s="10" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C176" s="11" t="s">
         <v>25</v>
@@ -5048,7 +5048,7 @@
         <v>10</v>
       </c>
       <c r="B177" s="10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C177" s="11" t="s">
         <v>25</v>
@@ -5065,7 +5065,7 @@
         <v>10</v>
       </c>
       <c r="B178" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C178" s="11" t="s">
         <v>25</v>
@@ -5082,7 +5082,7 @@
         <v>10</v>
       </c>
       <c r="B179" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C179" s="11" t="s">
         <v>25</v>
@@ -5099,7 +5099,7 @@
         <v>10</v>
       </c>
       <c r="B180" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C180" s="11" t="s">
         <v>25</v>
@@ -5116,7 +5116,7 @@
         <v>10</v>
       </c>
       <c r="B181" s="10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C181" s="11" t="s">
         <v>25</v>
@@ -5133,13 +5133,13 @@
         <v>10</v>
       </c>
       <c r="B182" s="10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C182" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D182" s="12" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E182" s="10" t="s">
         <v>27</v>
@@ -5150,7 +5150,7 @@
         <v>10</v>
       </c>
       <c r="B183" s="10" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C183" s="11" t="s">
         <v>25</v>
@@ -5167,7 +5167,7 @@
         <v>10</v>
       </c>
       <c r="B184" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C184" s="11" t="s">
         <v>25</v>
@@ -5184,7 +5184,7 @@
         <v>10</v>
       </c>
       <c r="B185" s="10" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C185" s="11" t="s">
         <v>25</v>
@@ -5201,7 +5201,7 @@
         <v>10</v>
       </c>
       <c r="B186" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C186" s="11" t="s">
         <v>25</v>
@@ -5218,7 +5218,7 @@
         <v>10</v>
       </c>
       <c r="B187" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C187" s="11" t="s">
         <v>25</v>
@@ -5235,7 +5235,7 @@
         <v>10</v>
       </c>
       <c r="B188" s="10" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C188" s="11" t="s">
         <v>25</v>
@@ -5252,7 +5252,7 @@
         <v>10</v>
       </c>
       <c r="B189" s="10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C189" s="11" t="s">
         <v>25</v>
@@ -5269,7 +5269,7 @@
         <v>10</v>
       </c>
       <c r="B190" s="10" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C190" s="11" t="s">
         <v>25</v>
@@ -5286,7 +5286,7 @@
         <v>10</v>
       </c>
       <c r="B191" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C191" s="11" t="s">
         <v>25</v>
@@ -5303,7 +5303,7 @@
         <v>10</v>
       </c>
       <c r="B192" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C192" s="11" t="s">
         <v>25</v>
@@ -5320,7 +5320,7 @@
         <v>10</v>
       </c>
       <c r="B193" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C193" s="11" t="s">
         <v>25</v>
@@ -5337,7 +5337,7 @@
         <v>10</v>
       </c>
       <c r="B194" s="10" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C194" s="11" t="s">
         <v>25</v>
@@ -5354,7 +5354,7 @@
         <v>10</v>
       </c>
       <c r="B195" s="10" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C195" s="11" t="s">
         <v>25</v>
@@ -5371,7 +5371,7 @@
         <v>10</v>
       </c>
       <c r="B196" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C196" s="11" t="s">
         <v>25</v>
@@ -5388,7 +5388,7 @@
         <v>10</v>
       </c>
       <c r="B197" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C197" s="11" t="s">
         <v>25</v>
@@ -5405,7 +5405,7 @@
         <v>10</v>
       </c>
       <c r="B198" s="10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C198" s="11" t="s">
         <v>25</v>
@@ -5422,7 +5422,7 @@
         <v>10</v>
       </c>
       <c r="B199" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C199" s="11" t="s">
         <v>25</v>
@@ -5439,7 +5439,7 @@
         <v>10</v>
       </c>
       <c r="B200" s="10" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C200" s="11" t="s">
         <v>25</v>
@@ -5456,7 +5456,7 @@
         <v>10</v>
       </c>
       <c r="B201" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C201" s="11" t="s">
         <v>25</v>
@@ -5473,7 +5473,7 @@
         <v>10</v>
       </c>
       <c r="B202" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C202" s="11" t="s">
         <v>25</v>
@@ -5490,7 +5490,7 @@
         <v>10</v>
       </c>
       <c r="B203" s="10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C203" s="11" t="s">
         <v>25</v>
@@ -5507,7 +5507,7 @@
         <v>10</v>
       </c>
       <c r="B204" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C204" s="11" t="s">
         <v>25</v>
@@ -5524,7 +5524,7 @@
         <v>10</v>
       </c>
       <c r="B205" s="10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C205" s="11" t="s">
         <v>25</v>
@@ -5541,7 +5541,7 @@
         <v>10</v>
       </c>
       <c r="B206" s="10" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C206" s="11" t="s">
         <v>25</v>
@@ -5558,7 +5558,7 @@
         <v>10</v>
       </c>
       <c r="B207" s="10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C207" s="11" t="s">
         <v>25</v>
@@ -5575,7 +5575,7 @@
         <v>10</v>
       </c>
       <c r="B208" s="10" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C208" s="11" t="s">
         <v>25</v>
@@ -5592,7 +5592,7 @@
         <v>10</v>
       </c>
       <c r="B209" s="10" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C209" s="11" t="s">
         <v>25</v>
@@ -5609,7 +5609,7 @@
         <v>10</v>
       </c>
       <c r="B210" s="10" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C210" s="11" t="s">
         <v>25</v>
@@ -5626,7 +5626,7 @@
         <v>10</v>
       </c>
       <c r="B211" s="10" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C211" s="11" t="s">
         <v>25</v>
@@ -5643,7 +5643,7 @@
         <v>10</v>
       </c>
       <c r="B212" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C212" s="11" t="s">
         <v>25</v>
@@ -5660,7 +5660,7 @@
         <v>10</v>
       </c>
       <c r="B213" s="10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C213" s="11" t="s">
         <v>25</v>
@@ -5677,7 +5677,7 @@
         <v>10</v>
       </c>
       <c r="B214" s="10" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C214" s="11" t="s">
         <v>25</v>
@@ -5694,7 +5694,7 @@
         <v>10</v>
       </c>
       <c r="B215" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C215" s="11" t="s">
         <v>25</v>
@@ -5711,7 +5711,7 @@
         <v>10</v>
       </c>
       <c r="B216" s="10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C216" s="11" t="s">
         <v>25</v>
@@ -5728,13 +5728,13 @@
         <v>10</v>
       </c>
       <c r="B217" s="10" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C217" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D217" s="12" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E217" s="10" t="s">
         <v>27</v>
@@ -5745,7 +5745,7 @@
         <v>10</v>
       </c>
       <c r="B218" s="10" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C218" s="11" t="s">
         <v>25</v>
@@ -5762,7 +5762,7 @@
         <v>10</v>
       </c>
       <c r="B219" s="10" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C219" s="11" t="s">
         <v>25</v>
@@ -5779,7 +5779,7 @@
         <v>10</v>
       </c>
       <c r="B220" s="10" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C220" s="11" t="s">
         <v>25</v>
@@ -5796,7 +5796,7 @@
         <v>10</v>
       </c>
       <c r="B221" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C221" s="11" t="s">
         <v>25</v>
@@ -5813,7 +5813,7 @@
         <v>12</v>
       </c>
       <c r="B222" s="10" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C222" s="11" t="s">
         <v>25</v>
@@ -5830,7 +5830,7 @@
         <v>12</v>
       </c>
       <c r="B223" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C223" s="11" t="s">
         <v>25</v>
@@ -5847,7 +5847,7 @@
         <v>12</v>
       </c>
       <c r="B224" s="10" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C224" s="11" t="s">
         <v>25</v>
@@ -5864,7 +5864,7 @@
         <v>12</v>
       </c>
       <c r="B225" s="10" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C225" s="11" t="s">
         <v>25</v>
@@ -5881,7 +5881,7 @@
         <v>12</v>
       </c>
       <c r="B226" s="10" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C226" s="11" t="s">
         <v>25</v>
@@ -5898,7 +5898,7 @@
         <v>12</v>
       </c>
       <c r="B227" s="10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C227" s="11" t="s">
         <v>25</v>
@@ -5915,7 +5915,7 @@
         <v>12</v>
       </c>
       <c r="B228" s="10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C228" s="11" t="s">
         <v>25</v>
@@ -5932,7 +5932,7 @@
         <v>12</v>
       </c>
       <c r="B229" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C229" s="11" t="s">
         <v>25</v>
@@ -5949,7 +5949,7 @@
         <v>12</v>
       </c>
       <c r="B230" s="10" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C230" s="11" t="s">
         <v>25</v>
@@ -5966,7 +5966,7 @@
         <v>12</v>
       </c>
       <c r="B231" s="10" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C231" s="11" t="s">
         <v>25</v>
@@ -5983,7 +5983,7 @@
         <v>12</v>
       </c>
       <c r="B232" s="10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C232" s="11" t="s">
         <v>25</v>
@@ -6000,7 +6000,7 @@
         <v>12</v>
       </c>
       <c r="B233" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C233" s="11" t="s">
         <v>25</v>
@@ -6017,7 +6017,7 @@
         <v>12</v>
       </c>
       <c r="B234" s="10" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C234" s="11" t="s">
         <v>25</v>
@@ -6034,7 +6034,7 @@
         <v>12</v>
       </c>
       <c r="B235" s="10" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C235" s="11" t="s">
         <v>25</v>
@@ -6051,7 +6051,7 @@
         <v>12</v>
       </c>
       <c r="B236" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C236" s="11" t="s">
         <v>25</v>
@@ -6068,7 +6068,7 @@
         <v>12</v>
       </c>
       <c r="B237" s="10" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C237" s="11" t="s">
         <v>25</v>
@@ -6085,7 +6085,7 @@
         <v>12</v>
       </c>
       <c r="B238" s="10" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C238" s="11" t="s">
         <v>25</v>
@@ -6102,7 +6102,7 @@
         <v>12</v>
       </c>
       <c r="B239" s="10" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C239" s="11" t="s">
         <v>25</v>
@@ -6119,7 +6119,7 @@
         <v>12</v>
       </c>
       <c r="B240" s="10" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C240" s="11" t="s">
         <v>25</v>
@@ -6136,7 +6136,7 @@
         <v>12</v>
       </c>
       <c r="B241" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C241" s="11" t="s">
         <v>25</v>
@@ -6153,7 +6153,7 @@
         <v>12</v>
       </c>
       <c r="B242" s="10" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C242" s="11" t="s">
         <v>25</v>
@@ -6170,7 +6170,7 @@
         <v>12</v>
       </c>
       <c r="B243" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C243" s="11" t="s">
         <v>25</v>
@@ -6187,7 +6187,7 @@
         <v>12</v>
       </c>
       <c r="B244" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C244" s="11" t="s">
         <v>25</v>
@@ -6204,7 +6204,7 @@
         <v>12</v>
       </c>
       <c r="B245" s="10" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C245" s="11" t="s">
         <v>25</v>
@@ -6221,7 +6221,7 @@
         <v>12</v>
       </c>
       <c r="B246" s="10" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C246" s="11" t="s">
         <v>25</v>
@@ -6238,7 +6238,7 @@
         <v>12</v>
       </c>
       <c r="B247" s="10" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C247" s="11" t="s">
         <v>25</v>
@@ -6255,7 +6255,7 @@
         <v>12</v>
       </c>
       <c r="B248" s="10" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C248" s="11" t="s">
         <v>25</v>
@@ -6272,7 +6272,7 @@
         <v>12</v>
       </c>
       <c r="B249" s="10" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C249" s="11" t="s">
         <v>25</v>
@@ -6289,7 +6289,7 @@
         <v>12</v>
       </c>
       <c r="B250" s="10" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C250" s="11" t="s">
         <v>25</v>
@@ -6306,7 +6306,7 @@
         <v>12</v>
       </c>
       <c r="B251" s="10" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C251" s="11" t="s">
         <v>25</v>
@@ -6323,7 +6323,7 @@
         <v>12</v>
       </c>
       <c r="B252" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C252" s="11" t="s">
         <v>25</v>
@@ -6340,7 +6340,7 @@
         <v>12</v>
       </c>
       <c r="B253" s="10" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C253" s="11" t="s">
         <v>25</v>
@@ -6357,7 +6357,7 @@
         <v>12</v>
       </c>
       <c r="B254" s="10" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C254" s="11" t="s">
         <v>25</v>
@@ -6374,7 +6374,7 @@
         <v>12</v>
       </c>
       <c r="B255" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C255" s="11" t="s">
         <v>25</v>
@@ -6391,7 +6391,7 @@
         <v>12</v>
       </c>
       <c r="B256" s="10" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C256" s="11" t="s">
         <v>25</v>
@@ -6408,7 +6408,7 @@
         <v>12</v>
       </c>
       <c r="B257" s="10" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C257" s="11" t="s">
         <v>25</v>
@@ -6425,7 +6425,7 @@
         <v>12</v>
       </c>
       <c r="B258" s="10" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C258" s="11" t="s">
         <v>25</v>
@@ -6442,7 +6442,7 @@
         <v>12</v>
       </c>
       <c r="B259" s="10" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C259" s="11" t="s">
         <v>25</v>
@@ -6459,7 +6459,7 @@
         <v>12</v>
       </c>
       <c r="B260" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C260" s="11" t="s">
         <v>25</v>
@@ -6476,7 +6476,7 @@
         <v>12</v>
       </c>
       <c r="B261" s="10" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C261" s="11" t="s">
         <v>25</v>
@@ -6493,7 +6493,7 @@
         <v>12</v>
       </c>
       <c r="B262" s="10" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C262" s="11" t="s">
         <v>25</v>
@@ -6510,7 +6510,7 @@
         <v>12</v>
       </c>
       <c r="B263" s="10" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C263" s="11" t="s">
         <v>25</v>
@@ -6527,7 +6527,7 @@
         <v>12</v>
       </c>
       <c r="B264" s="10" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C264" s="11" t="s">
         <v>25</v>
@@ -6544,7 +6544,7 @@
         <v>12</v>
       </c>
       <c r="B265" s="10" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C265" s="11" t="s">
         <v>25</v>
@@ -6561,7 +6561,7 @@
         <v>12</v>
       </c>
       <c r="B266" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C266" s="11" t="s">
         <v>25</v>
@@ -6578,7 +6578,7 @@
         <v>12</v>
       </c>
       <c r="B267" s="10" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C267" s="11" t="s">
         <v>25</v>
@@ -6595,7 +6595,7 @@
         <v>12</v>
       </c>
       <c r="B268" s="10" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C268" s="11" t="s">
         <v>25</v>
@@ -6612,7 +6612,7 @@
         <v>12</v>
       </c>
       <c r="B269" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C269" s="11" t="s">
         <v>25</v>
@@ -6629,7 +6629,7 @@
         <v>12</v>
       </c>
       <c r="B270" s="10" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C270" s="11" t="s">
         <v>25</v>
@@ -6646,7 +6646,7 @@
         <v>12</v>
       </c>
       <c r="B271" s="10" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C271" s="11" t="s">
         <v>25</v>
@@ -6663,7 +6663,7 @@
         <v>12</v>
       </c>
       <c r="B272" s="10" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C272" s="11" t="s">
         <v>25</v>
@@ -6680,7 +6680,7 @@
         <v>12</v>
       </c>
       <c r="B273" s="10" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C273" s="11" t="s">
         <v>25</v>
@@ -6697,7 +6697,7 @@
         <v>12</v>
       </c>
       <c r="B274" s="10" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C274" s="11" t="s">
         <v>25</v>
@@ -6714,7 +6714,7 @@
         <v>12</v>
       </c>
       <c r="B275" s="10" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C275" s="11" t="s">
         <v>25</v>
@@ -6731,7 +6731,7 @@
         <v>12</v>
       </c>
       <c r="B276" s="10" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C276" s="11" t="s">
         <v>25</v>
@@ -6748,7 +6748,7 @@
         <v>12</v>
       </c>
       <c r="B277" s="10" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C277" s="11" t="s">
         <v>25</v>
@@ -6765,7 +6765,7 @@
         <v>12</v>
       </c>
       <c r="B278" s="10" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C278" s="11" t="s">
         <v>25</v>
@@ -6782,7 +6782,7 @@
         <v>12</v>
       </c>
       <c r="B279" s="10" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C279" s="11" t="s">
         <v>25</v>
@@ -6799,7 +6799,7 @@
         <v>12</v>
       </c>
       <c r="B280" s="10" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C280" s="11" t="s">
         <v>25</v>
@@ -6816,7 +6816,7 @@
         <v>12</v>
       </c>
       <c r="B281" s="10" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C281" s="11" t="s">
         <v>25</v>
@@ -6833,7 +6833,7 @@
         <v>12</v>
       </c>
       <c r="B282" s="10" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C282" s="11" t="s">
         <v>25</v>
@@ -6850,7 +6850,7 @@
         <v>12</v>
       </c>
       <c r="B283" s="10" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C283" s="11" t="s">
         <v>25</v>
@@ -6867,7 +6867,7 @@
         <v>12</v>
       </c>
       <c r="B284" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C284" s="11" t="s">
         <v>25</v>
@@ -6884,7 +6884,7 @@
         <v>12</v>
       </c>
       <c r="B285" s="10" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C285" s="11" t="s">
         <v>25</v>
@@ -6901,7 +6901,7 @@
         <v>12</v>
       </c>
       <c r="B286" s="10" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C286" s="11" t="s">
         <v>25</v>
@@ -6918,7 +6918,7 @@
         <v>12</v>
       </c>
       <c r="B287" s="10" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C287" s="11" t="s">
         <v>25</v>
@@ -6935,7 +6935,7 @@
         <v>12</v>
       </c>
       <c r="B288" s="10" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C288" s="11" t="s">
         <v>25</v>
@@ -6952,7 +6952,7 @@
         <v>12</v>
       </c>
       <c r="B289" s="10" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C289" s="11" t="s">
         <v>25</v>
@@ -6969,7 +6969,7 @@
         <v>12</v>
       </c>
       <c r="B290" s="10" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C290" s="11" t="s">
         <v>25</v>
@@ -6986,7 +6986,7 @@
         <v>12</v>
       </c>
       <c r="B291" s="10" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C291" s="11" t="s">
         <v>25</v>
@@ -7003,7 +7003,7 @@
         <v>12</v>
       </c>
       <c r="B292" s="10" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C292" s="11" t="s">
         <v>25</v>
@@ -7020,7 +7020,7 @@
         <v>12</v>
       </c>
       <c r="B293" s="10" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C293" s="11" t="s">
         <v>25</v>
@@ -7037,7 +7037,7 @@
         <v>12</v>
       </c>
       <c r="B294" s="10" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C294" s="11" t="s">
         <v>25</v>
@@ -7054,7 +7054,7 @@
         <v>12</v>
       </c>
       <c r="B295" s="10" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C295" s="11" t="s">
         <v>25</v>
@@ -7071,7 +7071,7 @@
         <v>12</v>
       </c>
       <c r="B296" s="10" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C296" s="11" t="s">
         <v>25</v>
@@ -7088,7 +7088,7 @@
         <v>12</v>
       </c>
       <c r="B297" s="10" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C297" s="11" t="s">
         <v>25</v>
@@ -7105,7 +7105,7 @@
         <v>12</v>
       </c>
       <c r="B298" s="10" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C298" s="11" t="s">
         <v>25</v>
@@ -7122,7 +7122,7 @@
         <v>12</v>
       </c>
       <c r="B299" s="10" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C299" s="11" t="s">
         <v>25</v>
@@ -7139,7 +7139,7 @@
         <v>12</v>
       </c>
       <c r="B300" s="10" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C300" s="11" t="s">
         <v>25</v>
@@ -7156,7 +7156,7 @@
         <v>12</v>
       </c>
       <c r="B301" s="10" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C301" s="11" t="s">
         <v>25</v>
@@ -7173,7 +7173,7 @@
         <v>12</v>
       </c>
       <c r="B302" s="10" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C302" s="11" t="s">
         <v>25</v>
@@ -7190,7 +7190,7 @@
         <v>12</v>
       </c>
       <c r="B303" s="10" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C303" s="11" t="s">
         <v>25</v>
@@ -7207,7 +7207,7 @@
         <v>12</v>
       </c>
       <c r="B304" s="10" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C304" s="11" t="s">
         <v>25</v>
@@ -7224,7 +7224,7 @@
         <v>12</v>
       </c>
       <c r="B305" s="10" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C305" s="11" t="s">
         <v>25</v>
@@ -7241,7 +7241,7 @@
         <v>12</v>
       </c>
       <c r="B306" s="10" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C306" s="11" t="s">
         <v>25</v>
@@ -7258,7 +7258,7 @@
         <v>12</v>
       </c>
       <c r="B307" s="10" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C307" s="11" t="s">
         <v>25</v>
@@ -7275,7 +7275,7 @@
         <v>12</v>
       </c>
       <c r="B308" s="10" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C308" s="11" t="s">
         <v>25</v>
@@ -7292,7 +7292,7 @@
         <v>12</v>
       </c>
       <c r="B309" s="10" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C309" s="11" t="s">
         <v>25</v>
@@ -7309,7 +7309,7 @@
         <v>12</v>
       </c>
       <c r="B310" s="10" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C310" s="11" t="s">
         <v>25</v>
@@ -7326,7 +7326,7 @@
         <v>12</v>
       </c>
       <c r="B311" s="10" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C311" s="11" t="s">
         <v>25</v>
@@ -7343,7 +7343,7 @@
         <v>12</v>
       </c>
       <c r="B312" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C312" s="11" t="s">
         <v>25</v>
@@ -7360,7 +7360,7 @@
         <v>12</v>
       </c>
       <c r="B313" s="10" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C313" s="11" t="s">
         <v>25</v>
@@ -7377,7 +7377,7 @@
         <v>12</v>
       </c>
       <c r="B314" s="10" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C314" s="11" t="s">
         <v>25</v>
@@ -7394,7 +7394,7 @@
         <v>12</v>
       </c>
       <c r="B315" s="10" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C315" s="11" t="s">
         <v>25</v>
@@ -7411,7 +7411,7 @@
         <v>12</v>
       </c>
       <c r="B316" s="10" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C316" s="11" t="s">
         <v>25</v>
@@ -7428,7 +7428,7 @@
         <v>12</v>
       </c>
       <c r="B317" s="10" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C317" s="11" t="s">
         <v>25</v>
@@ -7445,7 +7445,7 @@
         <v>12</v>
       </c>
       <c r="B318" s="10" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C318" s="11" t="s">
         <v>25</v>
@@ -7462,7 +7462,7 @@
         <v>12</v>
       </c>
       <c r="B319" s="10" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C319" s="11" t="s">
         <v>25</v>
@@ -7479,7 +7479,7 @@
         <v>12</v>
       </c>
       <c r="B320" s="10" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C320" s="11" t="s">
         <v>25</v>
@@ -7496,7 +7496,7 @@
         <v>12</v>
       </c>
       <c r="B321" s="10" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C321" s="11" t="s">
         <v>25</v>
@@ -7513,13 +7513,13 @@
         <v>14</v>
       </c>
       <c r="B322" s="10" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C322" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D322" s="12" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E322" s="10" t="s">
         <v>27</v>
@@ -7530,13 +7530,13 @@
         <v>14</v>
       </c>
       <c r="B323" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="C323" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D323" s="12" t="s">
         <v>368</v>
-      </c>
-      <c r="C323" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="D323" s="12" t="s">
-        <v>369</v>
       </c>
       <c r="E323" s="10" t="s">
         <v>27</v>
@@ -7553,7 +7553,7 @@
         <v>25</v>
       </c>
       <c r="D324" s="12" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="E324" s="10" t="s">
         <v>27</v>
@@ -7564,13 +7564,13 @@
         <v>14</v>
       </c>
       <c r="B325" s="10" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C325" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D325" s="12" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E325" s="10" t="s">
         <v>27</v>
@@ -7581,13 +7581,13 @@
         <v>14</v>
       </c>
       <c r="B326" s="10" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C326" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D326" s="12" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="E326" s="10" t="s">
         <v>27</v>
@@ -7598,13 +7598,13 @@
         <v>14</v>
       </c>
       <c r="B327" s="10" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C327" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D327" s="12" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="E327" s="10" t="s">
         <v>27</v>
@@ -7615,13 +7615,13 @@
         <v>14</v>
       </c>
       <c r="B328" s="10" t="s">
+        <v>374</v>
+      </c>
+      <c r="C328" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D328" s="12" t="s">
         <v>375</v>
-      </c>
-      <c r="C328" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="D328" s="12" t="s">
-        <v>371</v>
       </c>
       <c r="E328" s="10" t="s">
         <v>27</v>
@@ -7638,7 +7638,7 @@
         <v>25</v>
       </c>
       <c r="D329" s="12" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="E329" s="10" t="s">
         <v>27</v>
@@ -7689,7 +7689,7 @@
         <v>25</v>
       </c>
       <c r="D332" s="12" t="s">
-        <v>371</v>
+        <v>380</v>
       </c>
       <c r="E332" s="10" t="s">
         <v>27</v>
@@ -7700,7 +7700,7 @@
         <v>14</v>
       </c>
       <c r="B333" s="10" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C333" s="11" t="s">
         <v>25</v>
@@ -7717,13 +7717,13 @@
         <v>14</v>
       </c>
       <c r="B334" s="10" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C334" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D334" s="12" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E334" s="10" t="s">
         <v>27</v>
@@ -7734,13 +7734,13 @@
         <v>14</v>
       </c>
       <c r="B335" s="10" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C335" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D335" s="12" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E335" s="10" t="s">
         <v>27</v>
@@ -7751,13 +7751,13 @@
         <v>14</v>
       </c>
       <c r="B336" s="10" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C336" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D336" s="12" t="s">
-        <v>371</v>
+        <v>380</v>
       </c>
       <c r="E336" s="10" t="s">
         <v>27</v>
@@ -7768,7 +7768,7 @@
         <v>14</v>
       </c>
       <c r="B337" s="10" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C337" s="11" t="s">
         <v>25</v>
@@ -7785,7 +7785,7 @@
         <v>14</v>
       </c>
       <c r="B338" s="10" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C338" s="11" t="s">
         <v>25</v>
@@ -7802,13 +7802,13 @@
         <v>14</v>
       </c>
       <c r="B339" s="10" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C339" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D339" s="12" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E339" s="10" t="s">
         <v>27</v>
@@ -7819,13 +7819,13 @@
         <v>14</v>
       </c>
       <c r="B340" s="10" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C340" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D340" s="12" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E340" s="10" t="s">
         <v>27</v>
@@ -7836,13 +7836,13 @@
         <v>14</v>
       </c>
       <c r="B341" s="10" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C341" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D341" s="12" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E341" s="10" t="s">
         <v>27</v>
@@ -7853,13 +7853,13 @@
         <v>14</v>
       </c>
       <c r="B342" s="10" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C342" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D342" s="12" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="E342" s="10" t="s">
         <v>27</v>
@@ -7870,7 +7870,7 @@
         <v>14</v>
       </c>
       <c r="B343" s="10" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C343" s="11" t="s">
         <v>25</v>
@@ -7887,13 +7887,13 @@
         <v>14</v>
       </c>
       <c r="B344" s="10" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C344" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D344" s="12" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="E344" s="10" t="s">
         <v>27</v>
@@ -7904,13 +7904,13 @@
         <v>14</v>
       </c>
       <c r="B345" s="10" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C345" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D345" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E345" s="10" t="s">
         <v>27</v>
@@ -7921,7 +7921,7 @@
         <v>14</v>
       </c>
       <c r="B346" s="10" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C346" s="11" t="s">
         <v>25</v>
@@ -7938,13 +7938,13 @@
         <v>14</v>
       </c>
       <c r="B347" s="10" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C347" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D347" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E347" s="10" t="s">
         <v>27</v>
@@ -7955,13 +7955,13 @@
         <v>14</v>
       </c>
       <c r="B348" s="10" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C348" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D348" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E348" s="10" t="s">
         <v>27</v>
@@ -7972,7 +7972,7 @@
         <v>14</v>
       </c>
       <c r="B349" s="10" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C349" s="11" t="s">
         <v>25</v>
@@ -7989,13 +7989,13 @@
         <v>14</v>
       </c>
       <c r="B350" s="10" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C350" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D350" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E350" s="10" t="s">
         <v>27</v>
@@ -8006,13 +8006,13 @@
         <v>14</v>
       </c>
       <c r="B351" s="10" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C351" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D351" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E351" s="10" t="s">
         <v>27</v>
@@ -8023,13 +8023,13 @@
         <v>14</v>
       </c>
       <c r="B352" s="10" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C352" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D352" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E352" s="10" t="s">
         <v>27</v>
@@ -8040,13 +8040,13 @@
         <v>14</v>
       </c>
       <c r="B353" s="10" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C353" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D353" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E353" s="10" t="s">
         <v>27</v>
@@ -8057,13 +8057,13 @@
         <v>14</v>
       </c>
       <c r="B354" s="10" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C354" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D354" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E354" s="10" t="s">
         <v>27</v>
@@ -8074,13 +8074,13 @@
         <v>14</v>
       </c>
       <c r="B355" s="10" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C355" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D355" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E355" s="10" t="s">
         <v>27</v>
@@ -8091,13 +8091,13 @@
         <v>14</v>
       </c>
       <c r="B356" s="10" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C356" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D356" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E356" s="10" t="s">
         <v>27</v>
@@ -8108,13 +8108,13 @@
         <v>14</v>
       </c>
       <c r="B357" s="10" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C357" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D357" s="12" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="E357" s="10" t="s">
         <v>27</v>
@@ -8125,13 +8125,13 @@
         <v>14</v>
       </c>
       <c r="B358" s="10" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C358" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D358" s="12" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="E358" s="10" t="s">
         <v>27</v>
@@ -8142,13 +8142,13 @@
         <v>14</v>
       </c>
       <c r="B359" s="10" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C359" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D359" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E359" s="10" t="s">
         <v>27</v>
@@ -8159,7 +8159,7 @@
         <v>14</v>
       </c>
       <c r="B360" s="10" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C360" s="11" t="s">
         <v>25</v>
@@ -8176,7 +8176,7 @@
         <v>14</v>
       </c>
       <c r="B361" s="10" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C361" s="11" t="s">
         <v>25</v>
@@ -8193,13 +8193,13 @@
         <v>14</v>
       </c>
       <c r="B362" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C362" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D362" s="12" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="E362" s="10" t="s">
         <v>27</v>
@@ -8210,13 +8210,13 @@
         <v>14</v>
       </c>
       <c r="B363" s="10" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C363" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D363" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E363" s="10" t="s">
         <v>27</v>
@@ -8227,7 +8227,7 @@
         <v>14</v>
       </c>
       <c r="B364" s="10" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C364" s="11" t="s">
         <v>25</v>
@@ -8244,13 +8244,13 @@
         <v>14</v>
       </c>
       <c r="B365" s="10" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C365" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D365" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E365" s="10" t="s">
         <v>27</v>
@@ -8261,13 +8261,13 @@
         <v>14</v>
       </c>
       <c r="B366" s="10" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C366" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D366" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E366" s="10" t="s">
         <v>27</v>
@@ -8278,13 +8278,13 @@
         <v>14</v>
       </c>
       <c r="B367" s="10" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C367" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D367" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E367" s="10" t="s">
         <v>27</v>
@@ -8295,13 +8295,13 @@
         <v>14</v>
       </c>
       <c r="B368" s="10" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C368" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D368" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E368" s="10" t="s">
         <v>27</v>
@@ -8312,13 +8312,13 @@
         <v>14</v>
       </c>
       <c r="B369" s="10" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C369" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D369" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E369" s="10" t="s">
         <v>27</v>
@@ -8329,13 +8329,13 @@
         <v>14</v>
       </c>
       <c r="B370" s="10" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C370" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D370" s="12" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="E370" s="10" t="s">
         <v>27</v>
@@ -8346,13 +8346,13 @@
         <v>14</v>
       </c>
       <c r="B371" s="10" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C371" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D371" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E371" s="10" t="s">
         <v>27</v>
@@ -8363,13 +8363,13 @@
         <v>14</v>
       </c>
       <c r="B372" s="10" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C372" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D372" s="12" t="s">
-        <v>420</v>
+        <v>70</v>
       </c>
       <c r="E372" s="10" t="s">
         <v>27</v>
@@ -8386,7 +8386,7 @@
         <v>25</v>
       </c>
       <c r="D373" s="12" t="s">
-        <v>420</v>
+        <v>29</v>
       </c>
       <c r="E373" s="10" t="s">
         <v>27</v>
@@ -8403,7 +8403,7 @@
         <v>25</v>
       </c>
       <c r="D374" s="12" t="s">
-        <v>140</v>
+        <v>70</v>
       </c>
       <c r="E374" s="10" t="s">
         <v>27</v>
@@ -8437,7 +8437,7 @@
         <v>25</v>
       </c>
       <c r="D376" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E376" s="10" t="s">
         <v>27</v>
@@ -8454,7 +8454,7 @@
         <v>25</v>
       </c>
       <c r="D377" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E377" s="10" t="s">
         <v>27</v>
@@ -8505,7 +8505,7 @@
         <v>25</v>
       </c>
       <c r="D380" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E380" s="10" t="s">
         <v>27</v>
@@ -8522,7 +8522,7 @@
         <v>25</v>
       </c>
       <c r="D381" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E381" s="10" t="s">
         <v>27</v>
@@ -8556,7 +8556,7 @@
         <v>25</v>
       </c>
       <c r="D383" s="12" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="E383" s="10" t="s">
         <v>27</v>
@@ -8573,7 +8573,7 @@
         <v>25</v>
       </c>
       <c r="D384" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E384" s="10" t="s">
         <v>27</v>
@@ -8590,7 +8590,7 @@
         <v>25</v>
       </c>
       <c r="D385" s="12" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="E385" s="10" t="s">
         <v>27</v>
@@ -8607,7 +8607,7 @@
         <v>25</v>
       </c>
       <c r="D386" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E386" s="10" t="s">
         <v>27</v>
@@ -8624,7 +8624,7 @@
         <v>25</v>
       </c>
       <c r="D387" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E387" s="10" t="s">
         <v>27</v>
@@ -8641,7 +8641,7 @@
         <v>25</v>
       </c>
       <c r="D388" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E388" s="10" t="s">
         <v>27</v>
@@ -8692,7 +8692,7 @@
         <v>25</v>
       </c>
       <c r="D391" s="12" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="E391" s="10" t="s">
         <v>27</v>
@@ -8709,7 +8709,7 @@
         <v>25</v>
       </c>
       <c r="D392" s="12" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="E392" s="10" t="s">
         <v>27</v>
@@ -8726,7 +8726,7 @@
         <v>25</v>
       </c>
       <c r="D393" s="12" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="E393" s="10" t="s">
         <v>27</v>
@@ -8743,7 +8743,7 @@
         <v>25</v>
       </c>
       <c r="D394" s="12" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="E394" s="10" t="s">
         <v>27</v>
@@ -8760,7 +8760,7 @@
         <v>25</v>
       </c>
       <c r="D395" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E395" s="10" t="s">
         <v>27</v>
@@ -8777,7 +8777,7 @@
         <v>25</v>
       </c>
       <c r="D396" s="12" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="E396" s="10" t="s">
         <v>27</v>
@@ -8811,7 +8811,7 @@
         <v>25</v>
       </c>
       <c r="D398" s="12" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="E398" s="10" t="s">
         <v>27</v>
@@ -8845,7 +8845,7 @@
         <v>25</v>
       </c>
       <c r="D400" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E400" s="10" t="s">
         <v>27</v>
@@ -8862,7 +8862,7 @@
         <v>25</v>
       </c>
       <c r="D401" s="12" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="E401" s="10" t="s">
         <v>27</v>
@@ -8879,7 +8879,7 @@
         <v>25</v>
       </c>
       <c r="D402" s="12" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="E402" s="10" t="s">
         <v>27</v>
@@ -8896,7 +8896,7 @@
         <v>25</v>
       </c>
       <c r="D403" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E403" s="10" t="s">
         <v>27</v>
@@ -8913,7 +8913,7 @@
         <v>25</v>
       </c>
       <c r="D404" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E404" s="10" t="s">
         <v>27</v>
@@ -8930,7 +8930,7 @@
         <v>25</v>
       </c>
       <c r="D405" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E405" s="10" t="s">
         <v>27</v>
@@ -8964,7 +8964,7 @@
         <v>25</v>
       </c>
       <c r="D407" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E407" s="10" t="s">
         <v>27</v>
@@ -8981,7 +8981,7 @@
         <v>25</v>
       </c>
       <c r="D408" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E408" s="10" t="s">
         <v>27</v>
@@ -8998,7 +8998,7 @@
         <v>25</v>
       </c>
       <c r="D409" s="12" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="E409" s="10" t="s">
         <v>27</v>
@@ -9015,7 +9015,7 @@
         <v>25</v>
       </c>
       <c r="D410" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E410" s="10" t="s">
         <v>27</v>
@@ -9032,7 +9032,7 @@
         <v>25</v>
       </c>
       <c r="D411" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E411" s="10" t="s">
         <v>27</v>
@@ -9066,7 +9066,7 @@
         <v>25</v>
       </c>
       <c r="D413" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E413" s="10" t="s">
         <v>27</v>
@@ -9083,7 +9083,7 @@
         <v>25</v>
       </c>
       <c r="D414" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E414" s="10" t="s">
         <v>27</v>
@@ -9100,7 +9100,7 @@
         <v>25</v>
       </c>
       <c r="D415" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E415" s="10" t="s">
         <v>27</v>
@@ -9117,7 +9117,7 @@
         <v>25</v>
       </c>
       <c r="D416" s="12" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E416" s="10" t="s">
         <v>27</v>
@@ -9134,7 +9134,7 @@
         <v>25</v>
       </c>
       <c r="D417" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E417" s="10" t="s">
         <v>27</v>
@@ -9168,7 +9168,7 @@
         <v>25</v>
       </c>
       <c r="D419" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E419" s="10" t="s">
         <v>27</v>
@@ -9185,7 +9185,7 @@
         <v>25</v>
       </c>
       <c r="D420" s="12" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E420" s="10" t="s">
         <v>27</v>
@@ -9202,7 +9202,7 @@
         <v>25</v>
       </c>
       <c r="D421" s="12" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="E421" s="10" t="s">
         <v>27</v>

</xml_diff>